<commit_message>
Ajusta ranking BP con métrica de peso bruto
Se renombra “participación abs.” a “peso bruto” en textos, encabezados, títulos y ayuda de CLI para aclarar la interpretación de las métricas en los rankings. Además, los rankings de participación y crecimiento ahora incluyen la columna de contribución (p.p.) y se ajusta el ancho de columnas en el Excel para mostrarla correctamente. También se actualizan los archivos de salida comparativos 2026Q2 vs 2026Q1 y 2026S1 vs 2025S1, y se agrega el documento BP_2026_2.docx.
</commit_message>
<xml_diff>
--- a/output/top_partidas_bp_2026Q2_vs_2026Q1.xlsx
+++ b/output/top_partidas_bp_2026Q2_vs_2026Q1.xlsx
@@ -450,7 +450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -494,33 +494,40 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Participación (%) = x_t / X_t. Con signos mixtos puede ser negativa o superar 100%; por eso el ranking de participación ordena por participación absoluta |x_t| / Σ|x_t|.</t>
+          <t>Participación (%) = x_t / X_t: peso de la partida sobre el SALDO NETO de la cuenta. Si hay partidas de signo contrario que se compensan, el neto es pequeño y la participación puede ser negativa o superar 100% (las participaciones suman 100%, pero mezclando positivos y negativos).</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Crecimiento (%) = (x_t − x_b) / |x_b|. Con saldos negativos, crecimiento positivo = el saldo sube (p. ej. menor déficit / menor salida neta).</t>
+          <t>Peso bruto (%) = |x_t| / Σ|x_t|: tamaño de la partida sobre la suma de los valores absolutos de todas las partidas (siempre entre 0 y 100%, suman 100%). El ranking de participación se ordena por esta medida. Peso bruto = |participación| × |X_t| / Σ|x_t|, así que la razón entre ambas es la misma para todas las partidas de una tabla.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Ranking de crecimiento: solo partidas con participación absoluta ≥ 1.0% en t o en b, para evitar crecimientos enormes de partidas con base casi nula.</t>
+          <t>Crecimiento (%) = (x_t − x_b) / |x_b|. Con saldos negativos, crecimiento positivo = el saldo sube (p. ej. menor déficit / menor salida neta).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Contribución (p.p.) = (x_t − x_b) / |X_b|; la suma de contribuciones es el crecimiento del total. Ranking por valor absoluto (el signo indica si empuja hacia arriba o hacia abajo).</t>
+          <t>Ranking de crecimiento: solo partidas con peso bruto ≥ 1.0% en t o en b, para evitar crecimientos enormes de partidas con base casi nula.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
+        <is>
+          <t>Contribución (p.p.) = (x_t − x_b) / |X_b|; la suma de contribuciones es el crecimiento del total. Ranking por valor absoluto (el signo indica si empuja hacia arriba o hacia abajo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t>Hoja 'Control': total oficial BanRep vs suma de partidas (debe ser ≈ 0).</t>
         </is>
@@ -537,7 +544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I28"/>
+  <dimension ref="A1:J28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -549,6 +556,7 @@
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -595,7 +603,7 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Participación abs. 2026Q2 (%)</t>
+          <t>Peso bruto 2026Q2 (%)</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -605,15 +613,20 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
+          <t>Contribución (p.p.)</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
           <t>Valor 2026Q2 (USD mill.)</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>Valor 2026Q1 (USD mill.)</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="J5" s="4" t="inlineStr">
         <is>
           <t>Variación (USD mill.)</t>
         </is>
@@ -643,12 +656,15 @@
         <v>-28.20952252551175</v>
       </c>
       <c r="G6" s="5" t="n">
+        <v>-111.6743130409039</v>
+      </c>
+      <c r="H6" s="5" t="n">
         <v>-6488.489704</v>
       </c>
-      <c r="H6" s="5" t="n">
+      <c r="I6" s="5" t="n">
         <v>-5060.848505</v>
       </c>
-      <c r="I6" s="5" t="n">
+      <c r="J6" s="5" t="n">
         <v>-1427.641199</v>
       </c>
     </row>
@@ -676,12 +692,15 @@
         <v>-0.3362802579075503</v>
       </c>
       <c r="G7" s="5" t="n">
+        <v>-0.8528488800552776</v>
+      </c>
+      <c r="H7" s="5" t="n">
         <v>3231.2725162</v>
       </c>
-      <c r="H7" s="5" t="n">
+      <c r="I7" s="5" t="n">
         <v>3242.1753117</v>
       </c>
-      <c r="I7" s="5" t="n">
+      <c r="J7" s="5" t="n">
         <v>-10.90279549999968</v>
       </c>
     </row>
@@ -709,12 +728,15 @@
         <v>-27.33496333013887</v>
       </c>
       <c r="G8" s="5" t="n">
+        <v>-46.29242312569009</v>
+      </c>
+      <c r="H8" s="5" t="n">
         <v>1573.19551</v>
       </c>
-      <c r="H8" s="5" t="n">
+      <c r="I8" s="5" t="n">
         <v>2164.9965129</v>
       </c>
-      <c r="I8" s="5" t="n">
+      <c r="J8" s="5" t="n">
         <v>-591.8010029000002</v>
       </c>
     </row>
@@ -742,12 +764,15 @@
         <v>-12.04898354565174</v>
       </c>
       <c r="G9" s="5" t="n">
+        <v>-11.14450784032718</v>
+      </c>
+      <c r="H9" s="5" t="n">
         <v>-1324.903315</v>
       </c>
-      <c r="H9" s="5" t="n">
+      <c r="I9" s="5" t="n">
         <v>-1182.432248</v>
       </c>
-      <c r="I9" s="5" t="n">
+      <c r="J9" s="5" t="n">
         <v>-142.4710669999999</v>
       </c>
     </row>
@@ -775,19 +800,22 @@
         <v>-8.625110673639082</v>
       </c>
       <c r="G10" s="5" t="n">
+        <v>-5.762115737482246</v>
+      </c>
+      <c r="H10" s="5" t="n">
         <v>-927.7123017</v>
       </c>
-      <c r="H10" s="5" t="n">
+      <c r="I10" s="5" t="n">
         <v>-854.0495802</v>
       </c>
-      <c r="I10" s="5" t="n">
+      <c r="J10" s="5" t="n">
         <v>-73.66272149999998</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Top 5 por crecimiento (partidas con participación abs. ≥ 1.0%)</t>
+          <t>Top 5 por crecimiento (partidas con peso bruto ≥ 1.0%)</t>
         </is>
       </c>
     </row>
@@ -819,20 +847,25 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Participación abs. 2026Q2 (%)</t>
+          <t>Peso bruto 2026Q2 (%)</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
+          <t>Contribución (p.p.)</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
           <t>Valor 2026Q2 (USD mill.)</t>
         </is>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>Valor 2026Q1 (USD mill.)</t>
         </is>
       </c>
-      <c r="I14" s="4" t="inlineStr">
+      <c r="J14" s="4" t="inlineStr">
         <is>
           <t>Variación (USD mill.)</t>
         </is>
@@ -862,12 +895,15 @@
         <v>1.009560877829699</v>
       </c>
       <c r="G15" s="5" t="n">
+        <v>2.862366873845029</v>
+      </c>
+      <c r="H15" s="5" t="n">
         <v>216.62143722</v>
       </c>
-      <c r="H15" s="5" t="n">
+      <c r="I15" s="5" t="n">
         <v>180.02902161</v>
       </c>
-      <c r="I15" s="5" t="n">
+      <c r="J15" s="5" t="n">
         <v>36.59241560999999</v>
       </c>
     </row>
@@ -895,12 +931,15 @@
         <v>2.774620182397185</v>
       </c>
       <c r="G16" s="5" t="n">
+        <v>1.699087649774975</v>
+      </c>
+      <c r="H16" s="5" t="n">
         <v>595.35014168</v>
       </c>
-      <c r="H16" s="5" t="n">
+      <c r="I16" s="5" t="n">
         <v>573.62905414</v>
       </c>
-      <c r="I16" s="5" t="n">
+      <c r="J16" s="5" t="n">
         <v>21.72108753999998</v>
       </c>
     </row>
@@ -928,12 +967,15 @@
         <v>2.101471290310967</v>
       </c>
       <c r="G17" s="5" t="n">
+        <v>0.6187512386550487</v>
+      </c>
+      <c r="H17" s="5" t="n">
         <v>-450.9126108</v>
       </c>
-      <c r="H17" s="5" t="n">
+      <c r="I17" s="5" t="n">
         <v>-458.8227088</v>
       </c>
-      <c r="I17" s="5" t="n">
+      <c r="J17" s="5" t="n">
         <v>7.910098000000005</v>
       </c>
     </row>
@@ -961,12 +1003,15 @@
         <v>15.05929588422409</v>
       </c>
       <c r="G18" s="5" t="n">
+        <v>-0.8528488800552776</v>
+      </c>
+      <c r="H18" s="5" t="n">
         <v>3231.2725162</v>
       </c>
-      <c r="H18" s="5" t="n">
+      <c r="I18" s="5" t="n">
         <v>3242.1753117</v>
       </c>
-      <c r="I18" s="5" t="n">
+      <c r="J18" s="5" t="n">
         <v>-10.90279549999968</v>
       </c>
     </row>
@@ -994,12 +1039,15 @@
         <v>1.070188975897139</v>
       </c>
       <c r="G19" s="5" t="n">
+        <v>-0.2021458406350111</v>
+      </c>
+      <c r="H19" s="5" t="n">
         <v>-229.6304058</v>
       </c>
-      <c r="H19" s="5" t="n">
+      <c r="I19" s="5" t="n">
         <v>-227.0461792</v>
       </c>
-      <c r="I19" s="5" t="n">
+      <c r="J19" s="5" t="n">
         <v>-2.584226599999994</v>
       </c>
     </row>
@@ -1233,7 +1281,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I28"/>
+  <dimension ref="A1:J28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1245,6 +1293,7 @@
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1291,7 +1340,7 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Participación abs. 2026Q2 (%)</t>
+          <t>Peso bruto 2026Q2 (%)</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -1301,15 +1350,20 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
+          <t>Contribución (p.p.)</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
           <t>Valor 2026Q2 (USD mill.)</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>Valor 2026Q1 (USD mill.)</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="J5" s="4" t="inlineStr">
         <is>
           <t>Variación (USD mill.)</t>
         </is>
@@ -1339,12 +1393,15 @@
         <v>8.225772618907481</v>
       </c>
       <c r="G6" s="5" t="n">
+        <v>3.676623234253844</v>
+      </c>
+      <c r="H6" s="5" t="n">
         <v>12789.087555</v>
       </c>
-      <c r="H6" s="5" t="n">
+      <c r="I6" s="5" t="n">
         <v>11817.044356</v>
       </c>
-      <c r="I6" s="5" t="n">
+      <c r="J6" s="5" t="n">
         <v>972.0431989999997</v>
       </c>
     </row>
@@ -1372,12 +1429,15 @@
         <v>-0.505018958220087</v>
       </c>
       <c r="G7" s="5" t="n">
+        <v>-0.06393256053133688</v>
+      </c>
+      <c r="H7" s="5" t="n">
         <v>3330.0597739</v>
       </c>
-      <c r="H7" s="5" t="n">
+      <c r="I7" s="5" t="n">
         <v>3346.9625694</v>
       </c>
-      <c r="I7" s="5" t="n">
+      <c r="J7" s="5" t="n">
         <v>-16.90279550000014</v>
       </c>
     </row>
@@ -1405,12 +1465,15 @@
         <v>-22.5652202653073</v>
       </c>
       <c r="G8" s="5" t="n">
+        <v>-2.281022215378539</v>
+      </c>
+      <c r="H8" s="5" t="n">
         <v>2069.4857668</v>
       </c>
-      <c r="H8" s="5" t="n">
+      <c r="I8" s="5" t="n">
         <v>2672.5533073</v>
       </c>
-      <c r="I8" s="5" t="n">
+      <c r="J8" s="5" t="n">
         <v>-603.0675405000002</v>
       </c>
     </row>
@@ -1438,12 +1501,15 @@
         <v>-27.33496333013887</v>
       </c>
       <c r="G9" s="5" t="n">
+        <v>-2.238408045604635</v>
+      </c>
+      <c r="H9" s="5" t="n">
         <v>1573.19551</v>
       </c>
-      <c r="H9" s="5" t="n">
+      <c r="I9" s="5" t="n">
         <v>2164.9965129</v>
       </c>
-      <c r="I9" s="5" t="n">
+      <c r="J9" s="5" t="n">
         <v>-591.8010029000002</v>
       </c>
     </row>
@@ -1471,19 +1537,22 @@
         <v>-6.149457268779948</v>
       </c>
       <c r="G10" s="5" t="n">
+        <v>-0.2225420032861977</v>
+      </c>
+      <c r="H10" s="5" t="n">
         <v>897.94230329</v>
       </c>
-      <c r="H10" s="5" t="n">
+      <c r="I10" s="5" t="n">
         <v>956.7790203</v>
       </c>
-      <c r="I10" s="5" t="n">
+      <c r="J10" s="5" t="n">
         <v>-58.83671700999992</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Top 5 por crecimiento (partidas con participación abs. ≥ 1.0%)</t>
+          <t>Top 5 por crecimiento (partidas con peso bruto ≥ 1.0%)</t>
         </is>
       </c>
     </row>
@@ -1515,20 +1584,25 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Participación abs. 2026Q2 (%)</t>
+          <t>Peso bruto 2026Q2 (%)</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
+          <t>Contribución (p.p.)</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
           <t>Valor 2026Q2 (USD mill.)</t>
         </is>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>Valor 2026Q1 (USD mill.)</t>
         </is>
       </c>
-      <c r="I14" s="4" t="inlineStr">
+      <c r="J14" s="4" t="inlineStr">
         <is>
           <t>Variación (USD mill.)</t>
         </is>
@@ -1558,12 +1632,15 @@
         <v>3.197657250694081</v>
       </c>
       <c r="G15" s="5" t="n">
+        <v>0.6153145961722597</v>
+      </c>
+      <c r="H15" s="5" t="n">
         <v>844.65848197</v>
       </c>
-      <c r="H15" s="5" t="n">
+      <c r="I15" s="5" t="n">
         <v>681.97867217</v>
       </c>
-      <c r="I15" s="5" t="n">
+      <c r="J15" s="5" t="n">
         <v>162.6798098</v>
       </c>
     </row>
@@ -1591,12 +1668,15 @@
         <v>1.823648494193881</v>
       </c>
       <c r="G16" s="5" t="n">
+        <v>0.3220433178920507</v>
+      </c>
+      <c r="H16" s="5" t="n">
         <v>481.71522086</v>
       </c>
-      <c r="H16" s="5" t="n">
+      <c r="I16" s="5" t="n">
         <v>396.57187138</v>
       </c>
-      <c r="I16" s="5" t="n">
+      <c r="J16" s="5" t="n">
         <v>85.14334947999998</v>
       </c>
     </row>
@@ -1624,12 +1704,15 @@
         <v>1.215486286844559</v>
       </c>
       <c r="G17" s="5" t="n">
+        <v>0.1777204744291864</v>
+      </c>
+      <c r="H17" s="5" t="n">
         <v>321.06968365</v>
       </c>
-      <c r="H17" s="5" t="n">
+      <c r="I17" s="5" t="n">
         <v>274.08309637</v>
       </c>
-      <c r="I17" s="5" t="n">
+      <c r="J17" s="5" t="n">
         <v>46.98658727999998</v>
       </c>
     </row>
@@ -1657,12 +1740,15 @@
         <v>48.41615803659173</v>
       </c>
       <c r="G18" s="5" t="n">
+        <v>3.676623234253844</v>
+      </c>
+      <c r="H18" s="5" t="n">
         <v>12789.087555</v>
       </c>
-      <c r="H18" s="5" t="n">
+      <c r="I18" s="5" t="n">
         <v>11817.044356</v>
       </c>
-      <c r="I18" s="5" t="n">
+      <c r="J18" s="5" t="n">
         <v>972.0431989999997</v>
       </c>
     </row>
@@ -1690,12 +1776,15 @@
         <v>2.558209977252485</v>
       </c>
       <c r="G19" s="5" t="n">
+        <v>0.1202785515804667</v>
+      </c>
+      <c r="H19" s="5" t="n">
         <v>675.74902078</v>
       </c>
-      <c r="H19" s="5" t="n">
+      <c r="I19" s="5" t="n">
         <v>643.94920323</v>
       </c>
-      <c r="I19" s="5" t="n">
+      <c r="J19" s="5" t="n">
         <v>31.79981755000006</v>
       </c>
     </row>
@@ -1929,7 +2018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I28"/>
+  <dimension ref="A1:J28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1941,6 +2030,7 @@
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1987,7 +2077,7 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Participación abs. 2026Q2 (%)</t>
+          <t>Peso bruto 2026Q2 (%)</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -1997,15 +2087,20 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
+          <t>Contribución (p.p.)</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
           <t>Valor 2026Q2 (USD mill.)</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>Valor 2026Q1 (USD mill.)</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="J5" s="4" t="inlineStr">
         <is>
           <t>Variación (USD mill.)</t>
         </is>
@@ -2035,12 +2130,15 @@
         <v>14.21791462810496</v>
       </c>
       <c r="G6" s="5" t="n">
+        <v>8.657846344036251</v>
+      </c>
+      <c r="H6" s="5" t="n">
         <v>19277.577259</v>
       </c>
-      <c r="H6" s="5" t="n">
+      <c r="I6" s="5" t="n">
         <v>16877.892861</v>
       </c>
-      <c r="I6" s="5" t="n">
+      <c r="J6" s="5" t="n">
         <v>2399.684398000001</v>
       </c>
     </row>
@@ -2068,12 +2166,15 @@
         <v>17.45331379794148</v>
       </c>
       <c r="G7" s="5" t="n">
+        <v>0.8663317007782223</v>
+      </c>
+      <c r="H7" s="5" t="n">
         <v>1615.9050481</v>
       </c>
-      <c r="H7" s="5" t="n">
+      <c r="I7" s="5" t="n">
         <v>1375.7849786</v>
       </c>
-      <c r="I7" s="5" t="n">
+      <c r="J7" s="5" t="n">
         <v>240.1200695</v>
       </c>
     </row>
@@ -2101,12 +2202,15 @@
         <v>5.708347362288857</v>
       </c>
       <c r="G8" s="5" t="n">
+        <v>0.3058497723751314</v>
+      </c>
+      <c r="H8" s="5" t="n">
         <v>1569.8252346</v>
       </c>
-      <c r="H8" s="5" t="n">
+      <c r="I8" s="5" t="n">
         <v>1485.0532373</v>
       </c>
-      <c r="I8" s="5" t="n">
+      <c r="J8" s="5" t="n">
         <v>84.77199729999984</v>
       </c>
     </row>
@@ -2134,12 +2238,15 @@
         <v>13.56675354515547</v>
       </c>
       <c r="G9" s="5" t="n">
+        <v>0.5583952558894681</v>
+      </c>
+      <c r="H9" s="5" t="n">
         <v>1295.5710928</v>
       </c>
-      <c r="H9" s="5" t="n">
+      <c r="I9" s="5" t="n">
         <v>1140.801381</v>
       </c>
-      <c r="I9" s="5" t="n">
+      <c r="J9" s="5" t="n">
         <v>154.7697118000001</v>
       </c>
     </row>
@@ -2167,19 +2274,22 @@
         <v>7.843641419570793</v>
       </c>
       <c r="G10" s="5" t="n">
+        <v>0.3013827715814075</v>
+      </c>
+      <c r="H10" s="5" t="n">
         <v>1148.5224506</v>
       </c>
-      <c r="H10" s="5" t="n">
+      <c r="I10" s="5" t="n">
         <v>1064.9885663</v>
       </c>
-      <c r="I10" s="5" t="n">
+      <c r="J10" s="5" t="n">
         <v>83.53388429999995</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Top 5 por crecimiento (partidas con participación abs. ≥ 1.0%)</t>
+          <t>Top 5 por crecimiento (partidas con peso bruto ≥ 1.0%)</t>
         </is>
       </c>
     </row>
@@ -2211,20 +2321,25 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Participación abs. 2026Q2 (%)</t>
+          <t>Peso bruto 2026Q2 (%)</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
+          <t>Contribución (p.p.)</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
           <t>Valor 2026Q2 (USD mill.)</t>
         </is>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>Valor 2026Q1 (USD mill.)</t>
         </is>
       </c>
-      <c r="I14" s="4" t="inlineStr">
+      <c r="J14" s="4" t="inlineStr">
         <is>
           <t>Variación (USD mill.)</t>
         </is>
@@ -2254,12 +2369,15 @@
         <v>2.712461489824054</v>
       </c>
       <c r="G15" s="5" t="n">
+        <v>0.7803931399739241</v>
+      </c>
+      <c r="H15" s="5" t="n">
         <v>844.0419916</v>
       </c>
-      <c r="H15" s="5" t="n">
+      <c r="I15" s="5" t="n">
         <v>627.74140507</v>
       </c>
-      <c r="I15" s="5" t="n">
+      <c r="J15" s="5" t="n">
         <v>216.3005865299999</v>
       </c>
     </row>
@@ -2287,12 +2405,15 @@
         <v>2.569445274932284</v>
       </c>
       <c r="G16" s="5" t="n">
+        <v>0.4845731705579261</v>
+      </c>
+      <c r="H16" s="5" t="n">
         <v>799.53935394</v>
       </c>
-      <c r="H16" s="5" t="n">
+      <c r="I16" s="5" t="n">
         <v>665.23081682</v>
       </c>
-      <c r="I16" s="5" t="n">
+      <c r="J16" s="5" t="n">
         <v>134.30853712</v>
       </c>
     </row>
@@ -2320,12 +2441,15 @@
         <v>5.192964636599172</v>
       </c>
       <c r="G17" s="5" t="n">
+        <v>0.8663317007782223</v>
+      </c>
+      <c r="H17" s="5" t="n">
         <v>1615.9050481</v>
       </c>
-      <c r="H17" s="5" t="n">
+      <c r="I17" s="5" t="n">
         <v>1375.7849786</v>
       </c>
-      <c r="I17" s="5" t="n">
+      <c r="J17" s="5" t="n">
         <v>240.1200695</v>
       </c>
     </row>
@@ -2353,12 +2477,15 @@
         <v>3.033863930982144</v>
       </c>
       <c r="G18" s="5" t="n">
+        <v>0.4457362807275124</v>
+      </c>
+      <c r="H18" s="5" t="n">
         <v>944.05342312</v>
       </c>
-      <c r="H18" s="5" t="n">
+      <c r="I18" s="5" t="n">
         <v>820.50925798</v>
       </c>
-      <c r="I18" s="5" t="n">
+      <c r="J18" s="5" t="n">
         <v>123.54416514</v>
       </c>
     </row>
@@ -2386,12 +2513,15 @@
         <v>61.95152190594572</v>
       </c>
       <c r="G19" s="5" t="n">
+        <v>8.657846344036251</v>
+      </c>
+      <c r="H19" s="5" t="n">
         <v>19277.577259</v>
       </c>
-      <c r="H19" s="5" t="n">
+      <c r="I19" s="5" t="n">
         <v>16877.892861</v>
       </c>
-      <c r="I19" s="5" t="n">
+      <c r="J19" s="5" t="n">
         <v>2399.684398000001</v>
       </c>
     </row>
@@ -2625,7 +2755,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I28"/>
+  <dimension ref="A1:J28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2637,6 +2767,7 @@
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2683,7 +2814,7 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Participación abs. 2026Q2 (%)</t>
+          <t>Peso bruto 2026Q2 (%)</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -2693,15 +2824,20 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
+          <t>Contribución (p.p.)</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
           <t>Valor 2026Q2 (USD mill.)</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>Valor 2026Q1 (USD mill.)</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="J5" s="4" t="inlineStr">
         <is>
           <t>Variación (USD mill.)</t>
         </is>
@@ -2731,12 +2867,15 @@
         <v>289.2135534057788</v>
       </c>
       <c r="G6" s="5" t="n">
+        <v>2515.325264917227</v>
+      </c>
+      <c r="H6" s="5" t="n">
         <v>8985.435783999999</v>
       </c>
-      <c r="H6" s="5" t="n">
+      <c r="I6" s="5" t="n">
         <v>-4748.8330631</v>
       </c>
-      <c r="I6" s="5" t="n">
+      <c r="J6" s="5" t="n">
         <v>13734.2688471</v>
       </c>
     </row>
@@ -2764,12 +2903,15 @@
         <v>-290.5262440120404</v>
       </c>
       <c r="G7" s="5" t="n">
+        <v>-1182.327676772122</v>
+      </c>
+      <c r="H7" s="5" t="n">
         <v>-4233.686383</v>
       </c>
-      <c r="H7" s="5" t="n">
+      <c r="I7" s="5" t="n">
         <v>2222.1014249</v>
       </c>
-      <c r="I7" s="5" t="n">
+      <c r="J7" s="5" t="n">
         <v>-6455.7878079</v>
       </c>
     </row>
@@ -2797,12 +2939,15 @@
         <v>-52.08525457644512</v>
       </c>
       <c r="G8" s="5" t="n">
+        <v>-149.9227558264621</v>
+      </c>
+      <c r="H8" s="5" t="n">
         <v>-2390.2936949</v>
       </c>
-      <c r="H8" s="5" t="n">
+      <c r="I8" s="5" t="n">
         <v>-1571.680109</v>
       </c>
-      <c r="I8" s="5" t="n">
+      <c r="J8" s="5" t="n">
         <v>-818.6135859000001</v>
       </c>
     </row>
@@ -2830,12 +2975,15 @@
         <v>-20686.31605757239</v>
       </c>
       <c r="G9" s="5" t="n">
+        <v>-388.6062074488717</v>
+      </c>
+      <c r="H9" s="5" t="n">
         <v>-2111.6240771</v>
       </c>
-      <c r="H9" s="5" t="n">
+      <c r="I9" s="5" t="n">
         <v>10.257416</v>
       </c>
-      <c r="I9" s="5" t="n">
+      <c r="J9" s="5" t="n">
         <v>-2121.8814931</v>
       </c>
     </row>
@@ -2863,19 +3011,22 @@
         <v>-5115.974567440379</v>
       </c>
       <c r="G10" s="5" t="n">
+        <v>-277.4341642094276</v>
+      </c>
+      <c r="H10" s="5" t="n">
         <v>-1485.245622</v>
       </c>
-      <c r="H10" s="5" t="n">
+      <c r="I10" s="5" t="n">
         <v>29.610310061</v>
       </c>
-      <c r="I10" s="5" t="n">
+      <c r="J10" s="5" t="n">
         <v>-1514.855932061</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Top 5 por crecimiento (partidas con participación abs. ≥ 1.0%)</t>
+          <t>Top 5 por crecimiento (partidas con peso bruto ≥ 1.0%)</t>
         </is>
       </c>
     </row>
@@ -2907,20 +3058,25 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Participación abs. 2026Q2 (%)</t>
+          <t>Peso bruto 2026Q2 (%)</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
+          <t>Contribución (p.p.)</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
           <t>Valor 2026Q2 (USD mill.)</t>
         </is>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>Valor 2026Q1 (USD mill.)</t>
         </is>
       </c>
-      <c r="I14" s="4" t="inlineStr">
+      <c r="J14" s="4" t="inlineStr">
         <is>
           <t>Variación (USD mill.)</t>
         </is>
@@ -2950,12 +3106,15 @@
         <v>27.6408748248096</v>
       </c>
       <c r="G15" s="5" t="n">
+        <v>2515.325264917227</v>
+      </c>
+      <c r="H15" s="5" t="n">
         <v>8985.435783999999</v>
       </c>
-      <c r="H15" s="5" t="n">
+      <c r="I15" s="5" t="n">
         <v>-4748.8330631</v>
       </c>
-      <c r="I15" s="5" t="n">
+      <c r="J15" s="5" t="n">
         <v>13734.2688471</v>
       </c>
     </row>
@@ -2983,12 +3142,15 @@
         <v>0.4871448999051082</v>
       </c>
       <c r="G16" s="5" t="n">
+        <v>117.1992687562432</v>
+      </c>
+      <c r="H16" s="5" t="n">
         <v>158.36001007</v>
       </c>
-      <c r="H16" s="5" t="n">
+      <c r="I16" s="5" t="n">
         <v>-481.575623</v>
       </c>
-      <c r="I16" s="5" t="n">
+      <c r="J16" s="5" t="n">
         <v>639.93563307</v>
       </c>
     </row>
@@ -3016,12 +3178,15 @@
         <v>0.1850570561127599</v>
       </c>
       <c r="G17" s="5" t="n">
+        <v>96.54195483224493</v>
+      </c>
+      <c r="H17" s="5" t="n">
         <v>60.15794741</v>
       </c>
-      <c r="H17" s="5" t="n">
+      <c r="I17" s="5" t="n">
         <v>-466.98388239</v>
       </c>
-      <c r="I17" s="5" t="n">
+      <c r="J17" s="5" t="n">
         <v>527.1418298</v>
       </c>
     </row>
@@ -3049,12 +3214,15 @@
         <v>0.04216041924654843</v>
       </c>
       <c r="G18" s="5" t="n">
+        <v>60.4374684732467</v>
+      </c>
+      <c r="H18" s="5" t="n">
         <v>13.70541787</v>
       </c>
-      <c r="H18" s="5" t="n">
+      <c r="I18" s="5" t="n">
         <v>-316.29740603</v>
       </c>
-      <c r="I18" s="5" t="n">
+      <c r="J18" s="5" t="n">
         <v>330.0028239</v>
       </c>
     </row>
@@ -3082,12 +3250,15 @@
         <v>0.02534701711928642</v>
       </c>
       <c r="G19" s="5" t="n">
+        <v>49.33068001611928</v>
+      </c>
+      <c r="H19" s="5" t="n">
         <v>8.2397534841</v>
       </c>
-      <c r="H19" s="5" t="n">
+      <c r="I19" s="5" t="n">
         <v>-261.1173874</v>
       </c>
-      <c r="I19" s="5" t="n">
+      <c r="J19" s="5" t="n">
         <v>269.3571408841</v>
       </c>
     </row>
@@ -3321,7 +3492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I28"/>
+  <dimension ref="A1:J28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -3333,6 +3504,7 @@
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3379,7 +3551,7 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Participación abs. 2026Q2 (%)</t>
+          <t>Peso bruto 2026Q2 (%)</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -3389,15 +3561,20 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
+          <t>Contribución (p.p.)</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
           <t>Valor 2026Q2 (USD mill.)</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>Valor 2026Q1 (USD mill.)</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="J5" s="4" t="inlineStr">
         <is>
           <t>Variación (USD mill.)</t>
         </is>
@@ -3427,12 +3604,15 @@
         <v>-290.5262440120404</v>
       </c>
       <c r="G6" s="5" t="n">
+        <v>-86.81637786448107</v>
+      </c>
+      <c r="H6" s="5" t="n">
         <v>-4233.686383</v>
       </c>
-      <c r="H6" s="5" t="n">
+      <c r="I6" s="5" t="n">
         <v>2222.1014249</v>
       </c>
-      <c r="I6" s="5" t="n">
+      <c r="J6" s="5" t="n">
         <v>-6455.7878079</v>
       </c>
     </row>
@@ -3460,12 +3640,15 @@
         <v>-5115.974567440379</v>
       </c>
       <c r="G7" s="5" t="n">
+        <v>-20.37153464788965</v>
+      </c>
+      <c r="H7" s="5" t="n">
         <v>-1485.245622</v>
       </c>
-      <c r="H7" s="5" t="n">
+      <c r="I7" s="5" t="n">
         <v>29.610310061</v>
       </c>
-      <c r="I7" s="5" t="n">
+      <c r="J7" s="5" t="n">
         <v>-1514.855932061</v>
       </c>
     </row>
@@ -3493,12 +3676,15 @@
         <v>-331.1860963111317</v>
       </c>
       <c r="G8" s="5" t="n">
+        <v>-28.42243693683088</v>
+      </c>
+      <c r="H8" s="5" t="n">
         <v>-1475.361724</v>
       </c>
-      <c r="H8" s="5" t="n">
+      <c r="I8" s="5" t="n">
         <v>638.17061127</v>
       </c>
-      <c r="I8" s="5" t="n">
+      <c r="J8" s="5" t="n">
         <v>-2113.53233527</v>
       </c>
     </row>
@@ -3526,12 +3712,15 @@
         <v>-320.9872631768285</v>
       </c>
       <c r="G9" s="5" t="n">
+        <v>-12.21387926861426</v>
+      </c>
+      <c r="H9" s="5" t="n">
         <v>-1191.193636</v>
       </c>
-      <c r="H9" s="5" t="n">
+      <c r="I9" s="5" t="n">
         <v>-282.9524169</v>
       </c>
-      <c r="I9" s="5" t="n">
+      <c r="J9" s="5" t="n">
         <v>-908.2412191</v>
       </c>
     </row>
@@ -3559,19 +3748,22 @@
         <v>-57.62495502893301</v>
       </c>
       <c r="G10" s="5" t="n">
+        <v>-15.84166560795249</v>
+      </c>
+      <c r="H10" s="5" t="n">
         <v>866.2594781</v>
       </c>
-      <c r="H10" s="5" t="n">
+      <c r="I10" s="5" t="n">
         <v>2044.2679853</v>
       </c>
-      <c r="I10" s="5" t="n">
+      <c r="J10" s="5" t="n">
         <v>-1178.0085072</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Top 5 por crecimiento (partidas con participación abs. ≥ 1.0%)</t>
+          <t>Top 5 por crecimiento (partidas con peso bruto ≥ 1.0%)</t>
         </is>
       </c>
     </row>
@@ -3603,20 +3795,25 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Participación abs. 2026Q2 (%)</t>
+          <t>Peso bruto 2026Q2 (%)</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
+          <t>Contribución (p.p.)</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
           <t>Valor 2026Q2 (USD mill.)</t>
         </is>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>Valor 2026Q1 (USD mill.)</t>
         </is>
       </c>
-      <c r="I14" s="4" t="inlineStr">
+      <c r="J14" s="4" t="inlineStr">
         <is>
           <t>Variación (USD mill.)</t>
         </is>
@@ -3646,12 +3843,15 @@
         <v>1.206691995705927</v>
       </c>
       <c r="G15" s="5" t="n">
+        <v>8.605749659486268</v>
+      </c>
+      <c r="H15" s="5" t="n">
         <v>158.36001007</v>
       </c>
-      <c r="H15" s="5" t="n">
+      <c r="I15" s="5" t="n">
         <v>-481.575623</v>
       </c>
-      <c r="I15" s="5" t="n">
+      <c r="J15" s="5" t="n">
         <v>639.93563307</v>
       </c>
     </row>
@@ -3679,12 +3879,15 @@
         <v>0.06278633457688244</v>
       </c>
       <c r="G16" s="5" t="n">
+        <v>3.622270746704894</v>
+      </c>
+      <c r="H16" s="5" t="n">
         <v>8.2397534841</v>
       </c>
-      <c r="H16" s="5" t="n">
+      <c r="I16" s="5" t="n">
         <v>-261.1173874</v>
       </c>
-      <c r="I16" s="5" t="n">
+      <c r="J16" s="5" t="n">
         <v>269.3571408841</v>
       </c>
     </row>
@@ -3712,12 +3915,15 @@
         <v>6.436237462019492</v>
       </c>
       <c r="G17" s="5" t="n">
+        <v>2.187691457460227</v>
+      </c>
+      <c r="H17" s="5" t="n">
         <v>844.65848197</v>
       </c>
-      <c r="H17" s="5" t="n">
+      <c r="I17" s="5" t="n">
         <v>681.97867217</v>
       </c>
-      <c r="I17" s="5" t="n">
+      <c r="J17" s="5" t="n">
         <v>162.6798098</v>
       </c>
     </row>
@@ -3745,12 +3951,15 @@
         <v>4.160394191532136</v>
       </c>
       <c r="G18" s="5" t="n">
+        <v>0.5523981417849763</v>
+      </c>
+      <c r="H18" s="5" t="n">
         <v>545.98859395</v>
       </c>
-      <c r="H18" s="5" t="n">
+      <c r="I18" s="5" t="n">
         <v>504.91149218</v>
       </c>
-      <c r="I18" s="5" t="n">
+      <c r="J18" s="5" t="n">
         <v>41.07710177000001</v>
       </c>
     </row>
@@ -3778,12 +3987,15 @@
         <v>2.441738738074223</v>
       </c>
       <c r="G19" s="5" t="n">
+        <v>-2.260008862605886</v>
+      </c>
+      <c r="H19" s="5" t="n">
         <v>320.44115029</v>
       </c>
-      <c r="H19" s="5" t="n">
+      <c r="I19" s="5" t="n">
         <v>488.49858392</v>
       </c>
-      <c r="I19" s="5" t="n">
+      <c r="J19" s="5" t="n">
         <v>-168.05743363</v>
       </c>
     </row>
@@ -4017,7 +4229,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I28"/>
+  <dimension ref="A1:J28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -4029,6 +4241,7 @@
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4075,7 +4288,7 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Participación abs. 2026Q2 (%)</t>
+          <t>Peso bruto 2026Q2 (%)</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -4085,15 +4298,20 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
+          <t>Contribución (p.p.)</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
           <t>Valor 2026Q2 (USD mill.)</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>Valor 2026Q1 (USD mill.)</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="J5" s="4" t="inlineStr">
         <is>
           <t>Variación (USD mill.)</t>
         </is>
@@ -4123,12 +4341,15 @@
         <v>-289.2135534057788</v>
       </c>
       <c r="G6" s="5" t="n">
+        <v>-172.0619718883344</v>
+      </c>
+      <c r="H6" s="5" t="n">
         <v>-8985.435783999999</v>
       </c>
-      <c r="H6" s="5" t="n">
+      <c r="I6" s="5" t="n">
         <v>4748.8330631</v>
       </c>
-      <c r="I6" s="5" t="n">
+      <c r="J6" s="5" t="n">
         <v>-13734.2688471</v>
       </c>
     </row>
@@ -4156,12 +4377,15 @@
         <v>52.08525457644512</v>
       </c>
       <c r="G7" s="5" t="n">
+        <v>10.25553448622607</v>
+      </c>
+      <c r="H7" s="5" t="n">
         <v>2390.2936949</v>
       </c>
-      <c r="H7" s="5" t="n">
+      <c r="I7" s="5" t="n">
         <v>1571.680109</v>
       </c>
-      <c r="I7" s="5" t="n">
+      <c r="J7" s="5" t="n">
         <v>818.6135859000001</v>
       </c>
     </row>
@@ -4189,12 +4413,15 @@
         <v>20686.31605757239</v>
       </c>
       <c r="G8" s="5" t="n">
+        <v>26.58278484866263</v>
+      </c>
+      <c r="H8" s="5" t="n">
         <v>2111.6240771</v>
       </c>
-      <c r="H8" s="5" t="n">
+      <c r="I8" s="5" t="n">
         <v>-10.257416</v>
       </c>
-      <c r="I8" s="5" t="n">
+      <c r="J8" s="5" t="n">
         <v>2121.8814931</v>
       </c>
     </row>
@@ -4222,12 +4449,15 @@
         <v>13.56675354515547</v>
       </c>
       <c r="G9" s="5" t="n">
+        <v>1.938944263969332</v>
+      </c>
+      <c r="H9" s="5" t="n">
         <v>1295.5710928</v>
       </c>
-      <c r="H9" s="5" t="n">
+      <c r="I9" s="5" t="n">
         <v>1140.801381</v>
       </c>
-      <c r="I9" s="5" t="n">
+      <c r="J9" s="5" t="n">
         <v>154.7697118000001</v>
       </c>
     </row>
@@ -4255,19 +4485,22 @@
         <v>-100</v>
       </c>
       <c r="G10" s="5" t="n">
+        <v>-6.263965479482564</v>
+      </c>
+      <c r="H10" s="5" t="n">
         <v>-1000</v>
-      </c>
-      <c r="H10" s="5" t="n">
-        <v>-500</v>
       </c>
       <c r="I10" s="5" t="n">
         <v>-500</v>
       </c>
+      <c r="J10" s="5" t="n">
+        <v>-500</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Top 5 por crecimiento (partidas con participación abs. ≥ 1.0%)</t>
+          <t>Top 5 por crecimiento (partidas con peso bruto ≥ 1.0%)</t>
         </is>
       </c>
     </row>
@@ -4299,20 +4532,25 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Participación abs. 2026Q2 (%)</t>
+          <t>Peso bruto 2026Q2 (%)</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
+          <t>Contribución (p.p.)</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
           <t>Valor 2026Q2 (USD mill.)</t>
         </is>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>Valor 2026Q1 (USD mill.)</t>
         </is>
       </c>
-      <c r="I14" s="4" t="inlineStr">
+      <c r="J14" s="4" t="inlineStr">
         <is>
           <t>Variación (USD mill.)</t>
         </is>
@@ -4342,12 +4580,15 @@
         <v>10.89347527430934</v>
       </c>
       <c r="G15" s="5" t="n">
+        <v>26.58278484866263</v>
+      </c>
+      <c r="H15" s="5" t="n">
         <v>2111.6240771</v>
       </c>
-      <c r="H15" s="5" t="n">
+      <c r="I15" s="5" t="n">
         <v>-10.257416</v>
       </c>
-      <c r="I15" s="5" t="n">
+      <c r="J15" s="5" t="n">
         <v>2121.8814931</v>
       </c>
     </row>
@@ -4375,12 +4616,15 @@
         <v>2.600727817190259</v>
       </c>
       <c r="G16" s="5" t="n">
+        <v>7.588679903116974</v>
+      </c>
+      <c r="H16" s="5" t="n">
         <v>504.13291796</v>
       </c>
-      <c r="H16" s="5" t="n">
+      <c r="I16" s="5" t="n">
         <v>-101.6079604</v>
       </c>
-      <c r="I16" s="5" t="n">
+      <c r="J16" s="5" t="n">
         <v>605.74087836</v>
       </c>
     </row>
@@ -4408,12 +4652,15 @@
         <v>2.693218017974732</v>
       </c>
       <c r="G17" s="5" t="n">
+        <v>5.528794777368029</v>
+      </c>
+      <c r="H17" s="5" t="n">
         <v>522.06149722</v>
       </c>
-      <c r="H17" s="5" t="n">
+      <c r="I17" s="5" t="n">
         <v>80.74402863900001</v>
       </c>
-      <c r="I17" s="5" t="n">
+      <c r="J17" s="5" t="n">
         <v>441.317468581</v>
       </c>
     </row>
@@ -4441,12 +4688,15 @@
         <v>1.83866228430327</v>
       </c>
       <c r="G18" s="5" t="n">
+        <v>6.086494088034319</v>
+      </c>
+      <c r="H18" s="5" t="n">
         <v>356.41183841</v>
       </c>
-      <c r="H18" s="5" t="n">
+      <c r="I18" s="5" t="n">
         <v>-129.422104</v>
       </c>
-      <c r="I18" s="5" t="n">
+      <c r="J18" s="5" t="n">
         <v>485.83394241</v>
       </c>
     </row>
@@ -4474,12 +4724,15 @@
         <v>2.186740031000242</v>
       </c>
       <c r="G19" s="5" t="n">
+        <v>8.487472143138547</v>
+      </c>
+      <c r="H19" s="5" t="n">
         <v>423.88427784</v>
       </c>
-      <c r="H19" s="5" t="n">
+      <c r="I19" s="5" t="n">
         <v>-253.5996715</v>
       </c>
-      <c r="I19" s="5" t="n">
+      <c r="J19" s="5" t="n">
         <v>677.48394934</v>
       </c>
     </row>
@@ -4773,7 +5026,7 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Participación abs. 2026Q2 (%)</t>
+          <t>Peso bruto 2026Q2 (%)</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">

</xml_diff>